<commit_message>
Fix Vercel blob storage with allowOverwrite and direct cloud sync
</commit_message>
<xml_diff>
--- a/data/credit_receipts.xlsx
+++ b/data/credit_receipts.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
   <si>
     <t>Rt. No.</t>
   </si>
@@ -124,10 +124,13 @@
     <t>2026-09-19</t>
   </si>
   <si>
-    <t>DEEPAK</t>
-  </si>
-  <si>
-    <t>ONE CRORE TWENTY THREE LAKH THIRTY FOUR THOUSAND FOUR HUNDRED FORTY FIVE RUPEES ONLY</t>
+    <t>Test Customer Cloud</t>
+  </si>
+  <si>
+    <t>Five Thousand Only</t>
+  </si>
+  <si>
+    <t>Cash</t>
   </si>
 </sst>
 </file>
@@ -715,7 +718,7 @@
         <v>37</v>
       </c>
       <c r="D9">
-        <v>12334445</v>
+        <v>5000</v>
       </c>
       <c r="E9" t="s">
         <v>38</v>
@@ -724,7 +727,7 @@
         <v>11</v>
       </c>
       <c r="G9" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>